<commit_message>
add empty context data for Pakistan
</commit_message>
<xml_diff>
--- a/data/context_data.xlsx
+++ b/data/context_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26130"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://oekoinstev.sharepoint.com/sites/AgoraPtXTool/Freigegebene Dokumente/General/Daten/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j.aschauer\nobackup\ptx-boa\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1977" documentId="13_ncr:1_{57048A87-158B-4EA5-9C6F-1E45CE5AC6D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C5531AED-DA45-42B4-8A26-2B539E8F88FB}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B69C056-AA8E-47A1-BE01-EFA89FDB04A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="3" xr2:uid="{D16C601B-E1D6-40C0-8CC1-80505BE1FBB6}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{D16C601B-E1D6-40C0-8CC1-80505BE1FBB6}"/>
   </bookViews>
   <sheets>
     <sheet name="certification_schemes" sheetId="6" r:id="rId1"/>
@@ -263,7 +263,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1104" uniqueCount="653">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1118" uniqueCount="655">
   <si>
     <t>topic</t>
   </si>
@@ -2429,6 +2429,12 @@
   <si>
     <t>**Certification scheme**
 Voluntary certification scheme based on German and European legislation. Its main certification mark is the label *GreenHydrogen*. Beyond the basic requirements, the scheme also formulates additional requirements. If these are met, the GreenHydrogen+ certification mark can be used, which proves in a broader assessment scope a product's GHG intensity belwo a set threshold. In general, the scheme allows hydrogen producers to demonstrate specific product characteristics that - also - fulfil the requirements set in the EU Renewable Energy Directive.</t>
+  </si>
+  <si>
+    <t>PAK</t>
+  </si>
+  <si>
+    <t>Pakistan</t>
   </si>
 </sst>
 </file>
@@ -2693,21 +2699,7 @@
     <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="76">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="0" tint="-4.9989318521683403E-2"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="34">
     <dxf>
       <fill>
         <patternFill>
@@ -2946,286 +2938,6 @@
         </patternFill>
       </fill>
     </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -3240,7 +2952,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink1.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="b_disclaimer"/>
@@ -5086,7 +4798,7 @@
 </file>
 
 <file path=xl/externalLinks/externalLink2.xml><?xml version="1.0" encoding="utf-8"?>
-<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" mc:Ignorable="x14">
+<externalLink xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xxl21="http://schemas.microsoft.com/office/spreadsheetml/2021/extlinks2021" mc:Ignorable="x14 xxl21">
   <externalBook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1">
     <sheetNames>
       <sheetName val="Sheet1"/>
@@ -5124,9 +4836,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -5164,7 +4876,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -5270,7 +4982,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -5412,7 +5124,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -6116,259 +5828,99 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="J4">
-    <cfRule type="cellIs" dxfId="75" priority="71" operator="equal">
+  <conditionalFormatting sqref="J4:J7">
+    <cfRule type="cellIs" dxfId="33" priority="51" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="74" priority="72" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="52" operator="equal">
+      <formula>"yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J11:J15">
+    <cfRule type="cellIs" dxfId="31" priority="5" operator="equal">
+      <formula>"no"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="30" priority="6" operator="equal">
+      <formula>"yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K6:K12">
+    <cfRule type="cellIs" dxfId="29" priority="21" operator="equal">
+      <formula>"no"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="28" priority="22" operator="equal">
+      <formula>"yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="K14:K15">
+    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+      <formula>"no"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="26" priority="4" operator="equal">
+      <formula>"yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L9:L10">
+    <cfRule type="cellIs" dxfId="25" priority="37" operator="equal">
+      <formula>"no"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="24" priority="38" operator="equal">
+      <formula>"yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L5:M6">
+    <cfRule type="cellIs" dxfId="23" priority="55" operator="equal">
+      <formula>"no"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="22" priority="56" operator="equal">
+      <formula>"yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L12:N12">
+    <cfRule type="cellIs" dxfId="21" priority="15" operator="equal">
+      <formula>"no"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="20" priority="16" operator="equal">
+      <formula>"yes"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N6">
+    <cfRule type="cellIs" dxfId="19" priority="53" operator="equal">
+      <formula>"no"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="18" priority="54" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O4">
-    <cfRule type="cellIs" dxfId="73" priority="69" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="69" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="72" priority="70" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L5">
-    <cfRule type="cellIs" dxfId="71" priority="65" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="70" priority="66" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M5">
-    <cfRule type="cellIs" dxfId="69" priority="63" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="68" priority="64" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J5:J6">
-    <cfRule type="cellIs" dxfId="67" priority="61" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="66" priority="62" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K6">
-    <cfRule type="cellIs" dxfId="65" priority="59" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="64" priority="60" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L6">
-    <cfRule type="cellIs" dxfId="63" priority="57" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="62" priority="58" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M6">
-    <cfRule type="cellIs" dxfId="61" priority="55" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="60" priority="56" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N6">
-    <cfRule type="cellIs" dxfId="59" priority="53" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="58" priority="54" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J7">
-    <cfRule type="cellIs" dxfId="57" priority="51" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="56" priority="52" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K7">
-    <cfRule type="cellIs" dxfId="55" priority="49" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="54" priority="50" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K8">
-    <cfRule type="cellIs" dxfId="53" priority="47" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="52" priority="48" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K9">
-    <cfRule type="cellIs" dxfId="51" priority="45" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="50" priority="46" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L9">
-    <cfRule type="cellIs" dxfId="49" priority="43" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="48" priority="44" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="70" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O9">
-    <cfRule type="cellIs" dxfId="47" priority="41" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="41" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="46" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="42" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K10">
-    <cfRule type="cellIs" dxfId="45" priority="39" operator="equal">
+  <conditionalFormatting sqref="O11:O12">
+    <cfRule type="cellIs" dxfId="13" priority="13" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="44" priority="40" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L10">
-    <cfRule type="cellIs" dxfId="43" priority="37" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="42" priority="38" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J11">
-    <cfRule type="cellIs" dxfId="41" priority="35" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="40" priority="36" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K11">
-    <cfRule type="cellIs" dxfId="39" priority="33" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="38" priority="34" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O11">
-    <cfRule type="cellIs" dxfId="37" priority="31" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="36" priority="32" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J12">
-    <cfRule type="cellIs" dxfId="35" priority="23" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="34" priority="24" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K12">
-    <cfRule type="cellIs" dxfId="33" priority="21" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="22" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L12">
-    <cfRule type="cellIs" dxfId="31" priority="19" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="20" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M12">
-    <cfRule type="cellIs" dxfId="29" priority="17" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="18" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N12">
-    <cfRule type="cellIs" dxfId="27" priority="15" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="16" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O12">
-    <cfRule type="cellIs" dxfId="25" priority="13" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="14" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J13">
-    <cfRule type="cellIs" dxfId="23" priority="11" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="12" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J14">
-    <cfRule type="cellIs" dxfId="21" priority="9" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="10" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K14">
-    <cfRule type="cellIs" dxfId="19" priority="7" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="8" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J15">
-    <cfRule type="cellIs" dxfId="17" priority="5" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="6" operator="equal">
-      <formula>"yes"</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K15">
-    <cfRule type="cellIs" dxfId="15" priority="3" operator="equal">
-      <formula>"no"</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="14" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O15">
-    <cfRule type="cellIs" dxfId="13" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7141,7 +6693,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66EF205A-9961-4EC2-AED6-DBC55BECEA90}">
   <sheetPr codeName="Sheet7"/>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="12.42578125" style="2" customWidth="1"/>
@@ -8103,75 +7655,75 @@
     </row>
     <row r="23" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="20" t="s">
-        <v>273</v>
+        <v>653</v>
       </c>
       <c r="B23" s="20" t="s">
-        <v>274</v>
-      </c>
-      <c r="C23" s="21">
-        <v>29291.660047894893</v>
-      </c>
-      <c r="D23" s="21">
-        <v>1887.6000000000001</v>
-      </c>
-      <c r="E23" s="20">
-        <v>1</v>
-      </c>
-      <c r="F23" s="20">
-        <v>0</v>
-      </c>
-      <c r="G23" s="20" t="s">
+        <v>654</v>
+      </c>
+      <c r="C23" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="H23" s="22" t="s">
+      <c r="D23" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="I23" s="23" t="s">
-        <v>623</v>
-      </c>
-      <c r="J23" s="20" t="s">
-        <v>313</v>
-      </c>
-      <c r="K23" s="20" t="s">
-        <v>318</v>
-      </c>
-      <c r="L23" s="20" t="s">
-        <v>319</v>
-      </c>
-      <c r="M23" s="20" t="s">
-        <v>326</v>
-      </c>
-      <c r="N23" s="20" t="s">
-        <v>325</v>
+      <c r="E23" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="F23" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="H23" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="I23" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="J23" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="K23" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="L23" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="M23" s="21" t="s">
+        <v>12</v>
+      </c>
+      <c r="N23" s="21" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="24" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="20" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B24" s="20" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C24" s="21">
-        <v>7559.5180291508068</v>
-      </c>
-      <c r="D24" s="21" t="s">
-        <v>250</v>
+        <v>29291.660047894893</v>
+      </c>
+      <c r="D24" s="21">
+        <v>1887.6000000000001</v>
       </c>
       <c r="E24" s="20">
+        <v>1</v>
+      </c>
+      <c r="F24" s="20">
         <v>0</v>
-      </c>
-      <c r="F24" s="20">
-        <v>1</v>
       </c>
       <c r="G24" s="20" t="s">
         <v>12</v>
       </c>
-      <c r="H24" s="22">
-        <v>129.84832399999999</v>
+      <c r="H24" s="22" t="s">
+        <v>12</v>
       </c>
       <c r="I24" s="23" t="s">
-        <v>624</v>
+        <v>623</v>
       </c>
       <c r="J24" s="20" t="s">
         <v>313</v>
@@ -8191,31 +7743,31 @@
     </row>
     <row r="25" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="20" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="B25" s="20" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C25" s="21">
-        <v>192895.02833307866</v>
-      </c>
-      <c r="D25" s="21">
-        <v>15445.300000000001</v>
+        <v>7559.5180291508068</v>
+      </c>
+      <c r="D25" s="21" t="s">
+        <v>250</v>
       </c>
       <c r="E25" s="20">
-        <v>23</v>
+        <v>0</v>
       </c>
       <c r="F25" s="20">
         <v>1</v>
       </c>
       <c r="G25" s="20" t="s">
-        <v>254</v>
-      </c>
-      <c r="H25" s="22" t="s">
         <v>12</v>
       </c>
+      <c r="H25" s="22">
+        <v>129.84832399999999</v>
+      </c>
       <c r="I25" s="23" t="s">
-        <v>625</v>
+        <v>624</v>
       </c>
       <c r="J25" s="20" t="s">
         <v>313</v>
@@ -8235,31 +7787,31 @@
     </row>
     <row r="26" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="20" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="B26" s="20" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="C26" s="21">
-        <v>151622.74756959747</v>
+        <v>192895.02833307866</v>
       </c>
       <c r="D26" s="21">
-        <v>3477.5</v>
+        <v>15445.300000000001</v>
       </c>
       <c r="E26" s="20">
-        <v>0</v>
+        <v>23</v>
       </c>
       <c r="F26" s="20">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G26" s="20" t="s">
-        <v>236</v>
+        <v>254</v>
       </c>
       <c r="H26" s="22" t="s">
         <v>12</v>
       </c>
       <c r="I26" s="23" t="s">
-        <v>626</v>
+        <v>625</v>
       </c>
       <c r="J26" s="20" t="s">
         <v>313</v>
@@ -8279,22 +7831,22 @@
     </row>
     <row r="27" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="20" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="B27" s="20" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C27" s="21">
-        <v>53182.742412075226</v>
+        <v>151622.74756959747</v>
       </c>
       <c r="D27" s="21">
-        <v>1115.4000000000001</v>
+        <v>3477.5</v>
       </c>
       <c r="E27" s="20">
         <v>0</v>
       </c>
       <c r="F27" s="20">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G27" s="20" t="s">
         <v>236</v>
@@ -8303,7 +7855,7 @@
         <v>12</v>
       </c>
       <c r="I27" s="23" t="s">
-        <v>627</v>
+        <v>626</v>
       </c>
       <c r="J27" s="20" t="s">
         <v>313</v>
@@ -8323,31 +7875,31 @@
     </row>
     <row r="28" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="20" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="B28" s="20" t="s">
-        <v>6</v>
+        <v>282</v>
       </c>
       <c r="C28" s="21">
-        <v>35393.799778929817</v>
-      </c>
-      <c r="D28" s="21" t="s">
-        <v>250</v>
+        <v>53182.742412075226</v>
+      </c>
+      <c r="D28" s="21">
+        <v>1115.4000000000001</v>
       </c>
       <c r="E28" s="20">
         <v>0</v>
       </c>
       <c r="F28" s="20">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="G28" s="20" t="s">
+        <v>236</v>
+      </c>
+      <c r="H28" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="H28" s="22">
-        <v>122.662285</v>
-      </c>
       <c r="I28" s="23" t="s">
-        <v>628</v>
+        <v>627</v>
       </c>
       <c r="J28" s="20" t="s">
         <v>313</v>
@@ -8367,13 +7919,13 @@
     </row>
     <row r="29" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="20" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="B29" s="20" t="s">
-        <v>285</v>
+        <v>6</v>
       </c>
       <c r="C29" s="21">
-        <v>2375.3911489586781</v>
+        <v>35393.799778929817</v>
       </c>
       <c r="D29" s="21" t="s">
         <v>250</v>
@@ -8382,16 +7934,16 @@
         <v>0</v>
       </c>
       <c r="F29" s="20">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="G29" s="20" t="s">
-        <v>231</v>
+        <v>12</v>
       </c>
       <c r="H29" s="22">
-        <v>70.495289999999997</v>
+        <v>122.662285</v>
       </c>
       <c r="I29" s="23" t="s">
-        <v>629</v>
+        <v>628</v>
       </c>
       <c r="J29" s="20" t="s">
         <v>313</v>
@@ -8411,31 +7963,31 @@
     </row>
     <row r="30" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="20" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="B30" s="20" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C30" s="21">
-        <v>6534.4815097404735</v>
+        <v>2375.3911489586781</v>
       </c>
       <c r="D30" s="21" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="E30" s="20">
         <v>0</v>
       </c>
       <c r="F30" s="20">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="G30" s="20" t="s">
         <v>231</v>
       </c>
-      <c r="H30" s="22" t="s">
-        <v>12</v>
+      <c r="H30" s="22">
+        <v>70.495289999999997</v>
       </c>
       <c r="I30" s="23" t="s">
-        <v>630</v>
+        <v>629</v>
       </c>
       <c r="J30" s="20" t="s">
         <v>313</v>
@@ -8455,31 +8007,31 @@
     </row>
     <row r="31" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="20" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="B31" s="20" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C31" s="21">
-        <v>17975.881159055345</v>
-      </c>
-      <c r="D31" s="21">
-        <v>500.5</v>
+        <v>6534.4815097404735</v>
+      </c>
+      <c r="D31" s="21" t="s">
+        <v>245</v>
       </c>
       <c r="E31" s="20">
         <v>0</v>
       </c>
       <c r="F31" s="20">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="G31" s="20" t="s">
-        <v>12</v>
+        <v>231</v>
       </c>
       <c r="H31" s="22" t="s">
         <v>12</v>
       </c>
       <c r="I31" s="23" t="s">
-        <v>631</v>
+        <v>630</v>
       </c>
       <c r="J31" s="20" t="s">
         <v>313</v>
@@ -8499,31 +8051,31 @@
     </row>
     <row r="32" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="20" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="B32" s="20" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C32" s="21">
-        <v>1234.3228021367959</v>
+        <v>17975.881159055345</v>
       </c>
       <c r="D32" s="21">
-        <v>842.4</v>
+        <v>500.5</v>
       </c>
       <c r="E32" s="20">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="F32" s="20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G32" s="20" t="s">
-        <v>254</v>
+        <v>12</v>
       </c>
       <c r="H32" s="22" t="s">
         <v>12</v>
       </c>
       <c r="I32" s="23" t="s">
-        <v>632</v>
+        <v>631</v>
       </c>
       <c r="J32" s="20" t="s">
         <v>313</v>
@@ -8543,22 +8095,22 @@
     </row>
     <row r="33" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="20" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="B33" s="20" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C33" s="21">
-        <v>9001.3629494330653</v>
+        <v>1234.3228021367959</v>
       </c>
       <c r="D33" s="21">
-        <v>16.900000000000002</v>
+        <v>842.4</v>
       </c>
       <c r="E33" s="20">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="F33" s="20">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="G33" s="20" t="s">
         <v>254</v>
@@ -8567,7 +8119,7 @@
         <v>12</v>
       </c>
       <c r="I33" s="23" t="s">
-        <v>633</v>
+        <v>632</v>
       </c>
       <c r="J33" s="20" t="s">
         <v>313</v>
@@ -8587,16 +8139,16 @@
     </row>
     <row r="34" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="20" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="B34" s="20" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C34" s="21">
-        <v>378.04871500147641</v>
+        <v>9001.3629494330653</v>
       </c>
       <c r="D34" s="21">
-        <v>1280.5</v>
+        <v>16.900000000000002</v>
       </c>
       <c r="E34" s="20">
         <v>0</v>
@@ -8605,16 +8157,16 @@
         <v>0</v>
       </c>
       <c r="G34" s="20" t="s">
-        <v>12</v>
+        <v>254</v>
       </c>
       <c r="H34" s="22" t="s">
         <v>12</v>
       </c>
       <c r="I34" s="23" t="s">
-        <v>634</v>
+        <v>633</v>
       </c>
       <c r="J34" s="20" t="s">
-        <v>315</v>
+        <v>313</v>
       </c>
       <c r="K34" s="20" t="s">
         <v>318</v>
@@ -8631,34 +8183,34 @@
     </row>
     <row r="35" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="20" t="s">
-        <v>11</v>
+        <v>294</v>
       </c>
       <c r="B35" s="20" t="s">
-        <v>11</v>
+        <v>295</v>
       </c>
       <c r="C35" s="21">
-        <v>544110.99319185445</v>
+        <v>378.04871500147641</v>
       </c>
       <c r="D35" s="21">
-        <v>41844.400000000001</v>
+        <v>1280.5</v>
       </c>
       <c r="E35" s="20">
-        <v>124</v>
+        <v>0</v>
       </c>
       <c r="F35" s="20">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="G35" s="20" t="s">
-        <v>239</v>
-      </c>
-      <c r="H35" s="22">
-        <v>68.122753000000003</v>
+        <v>12</v>
+      </c>
+      <c r="H35" s="22" t="s">
+        <v>12</v>
       </c>
       <c r="I35" s="23" t="s">
-        <v>635</v>
+        <v>634</v>
       </c>
       <c r="J35" s="20" t="s">
-        <v>313</v>
+        <v>315</v>
       </c>
       <c r="K35" s="20" t="s">
         <v>318</v>
@@ -8675,31 +8227,31 @@
     </row>
     <row r="36" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="20" t="s">
-        <v>296</v>
+        <v>11</v>
       </c>
       <c r="B36" s="20" t="s">
-        <v>297</v>
+        <v>11</v>
       </c>
       <c r="C36" s="21">
-        <v>8842.3521510548053</v>
-      </c>
-      <c r="D36" s="21" t="s">
-        <v>245</v>
+        <v>544110.99319185445</v>
+      </c>
+      <c r="D36" s="21">
+        <v>41844.400000000001</v>
       </c>
       <c r="E36" s="20">
-        <v>0</v>
+        <v>124</v>
       </c>
       <c r="F36" s="20">
-        <v>20</v>
+        <v>8</v>
       </c>
       <c r="G36" s="20" t="s">
-        <v>254</v>
-      </c>
-      <c r="H36" s="22" t="s">
-        <v>12</v>
+        <v>239</v>
+      </c>
+      <c r="H36" s="22">
+        <v>68.122753000000003</v>
       </c>
       <c r="I36" s="23" t="s">
-        <v>636</v>
+        <v>635</v>
       </c>
       <c r="J36" s="20" t="s">
         <v>313</v>
@@ -8717,49 +8269,77 @@
         <v>325</v>
       </c>
     </row>
-    <row r="37" spans="1:14" x14ac:dyDescent="0.25">
-      <c r="C37" s="1"/>
-      <c r="D37" s="1"/>
-      <c r="E37" s="1"/>
-      <c r="F37" s="1"/>
-      <c r="G37" s="1"/>
-    </row>
-    <row r="38" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A38" s="16"/>
-      <c r="B38" s="16"/>
-      <c r="C38" s="17"/>
-      <c r="D38" s="17"/>
-      <c r="E38" s="17"/>
-      <c r="F38" s="17"/>
-      <c r="G38" s="17"/>
-      <c r="H38" s="17"/>
-      <c r="I38" s="15"/>
+    <row r="37" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="20" t="s">
+        <v>296</v>
+      </c>
+      <c r="B37" s="20" t="s">
+        <v>297</v>
+      </c>
+      <c r="C37" s="21">
+        <v>8842.3521510548053</v>
+      </c>
+      <c r="D37" s="21" t="s">
+        <v>245</v>
+      </c>
+      <c r="E37" s="20">
+        <v>0</v>
+      </c>
+      <c r="F37" s="20">
+        <v>20</v>
+      </c>
+      <c r="G37" s="20" t="s">
+        <v>254</v>
+      </c>
+      <c r="H37" s="22" t="s">
+        <v>12</v>
+      </c>
+      <c r="I37" s="23" t="s">
+        <v>636</v>
+      </c>
+      <c r="J37" s="20" t="s">
+        <v>313</v>
+      </c>
+      <c r="K37" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="L37" s="20" t="s">
+        <v>319</v>
+      </c>
+      <c r="M37" s="20" t="s">
+        <v>326</v>
+      </c>
+      <c r="N37" s="20" t="s">
+        <v>325</v>
+      </c>
     </row>
     <row r="39" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="16"/>
       <c r="B39" s="16"/>
       <c r="C39" s="17"/>
       <c r="D39" s="17"/>
-      <c r="E39" s="1"/>
-      <c r="F39" s="1"/>
+      <c r="E39" s="17"/>
+      <c r="F39" s="17"/>
       <c r="G39" s="17"/>
-      <c r="H39" s="18"/>
+      <c r="H39" s="17"/>
       <c r="I39" s="15"/>
     </row>
     <row r="40" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A40" s="16"/>
+      <c r="B40" s="16"/>
       <c r="C40" s="17"/>
       <c r="D40" s="17"/>
-    </row>
-    <row r="41" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="42" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="C42" s="17"/>
-      <c r="D42" s="17"/>
-      <c r="E42" s="17"/>
-      <c r="F42" s="17"/>
-      <c r="G42" s="17"/>
-      <c r="H42" s="17"/>
-      <c r="I42" s="17"/>
-    </row>
+      <c r="E40" s="1"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="17"/>
+      <c r="H40" s="18"/>
+      <c r="I40" s="15"/>
+    </row>
+    <row r="41" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C41" s="17"/>
+      <c r="D41" s="17"/>
+    </row>
+    <row r="42" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="43" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C43" s="17"/>
       <c r="D43" s="17"/>
@@ -8769,13 +8349,30 @@
       <c r="H43" s="17"/>
       <c r="I43" s="17"/>
     </row>
+    <row r="44" spans="1:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C44" s="17"/>
+      <c r="D44" s="17"/>
+      <c r="E44" s="17"/>
+      <c r="F44" s="17"/>
+      <c r="G44" s="17"/>
+      <c r="H44" s="17"/>
+      <c r="I44" s="17"/>
+    </row>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D3:D36">
-    <cfRule type="colorScale" priority="10">
+  <conditionalFormatting sqref="D3:D22 D24:D37">
+    <cfRule type="colorScale" priority="18">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8784,8 +8381,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F3:F36">
-    <cfRule type="colorScale" priority="9">
+  <conditionalFormatting sqref="E3:E22 E24:E37">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8794,8 +8391,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E3:E36">
-    <cfRule type="colorScale" priority="8">
+  <conditionalFormatting sqref="F3:F22 F24:F37">
+    <cfRule type="colorScale" priority="20">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8804,18 +8401,22 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D36">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
+  <conditionalFormatting sqref="G3:G37">
+    <cfRule type="cellIs" dxfId="9" priority="12" operator="equal">
+      <formula>"very high"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="8" priority="13" operator="equal">
+      <formula>"high"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="14" operator="equal">
+      <formula>"medium"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="15" operator="equal">
+      <formula>"low"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H3:H36">
-    <cfRule type="colorScale" priority="6">
+  <conditionalFormatting sqref="H3:H22 H24:H37">
+    <cfRule type="colorScale" priority="17">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -8826,7 +8427,67 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C36">
+  <conditionalFormatting sqref="D23">
+    <cfRule type="colorScale" priority="11">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E23">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F23">
+    <cfRule type="colorScale" priority="9">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G23">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="H23">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="I23">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J23">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -8836,18 +8497,54 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G3:G36">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
-      <formula>"very high"</formula>
+  <conditionalFormatting sqref="K23">
+    <cfRule type="colorScale" priority="4">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
-      <formula>"high"</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="L23">
+    <cfRule type="colorScale" priority="3">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
     </cfRule>
-    <cfRule type="cellIs" dxfId="9" priority="3" operator="equal">
-      <formula>"medium"</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="M23">
+    <cfRule type="colorScale" priority="2">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="4" operator="equal">
-      <formula>"low"</formula>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="N23">
+    <cfRule type="colorScale" priority="1">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="C3:C37">
+    <cfRule type="colorScale" priority="71">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
     </cfRule>
   </conditionalFormatting>
   <hyperlinks>
@@ -8871,20 +8568,20 @@
     <hyperlink ref="I20" r:id="rId18" display="https://www.mem.gov.ma/pages/actualite.aspx?act=278" xr:uid="{6C8DAB63-4F23-4C92-BDF4-154465B0C551}"/>
     <hyperlink ref="I21" r:id="rId19" display="https://www.energymonitor.ai/tech/hydrogen/namibia-stakes-its-future-on-the-green-hydrogen-market" xr:uid="{52C53890-B03B-4D93-BAC2-A32DD86D7BB1}"/>
     <hyperlink ref="I22" r:id="rId20" display="https://www.regjeringen.no/contentassets/8ffd54808d7e42e8bce81340b13b6b7d/hydrogenstrategien-engelsk.pdf" xr:uid="{F3E54031-18D0-4285-A49D-EF61966D52A7}"/>
-    <hyperlink ref="I23" r:id="rId21" display="https://fuelcellsworks.com/news/h2-peru-publishes-its-proposal-for-a-green-hydrogen-roadmap-in-peru/" xr:uid="{93D8A6AB-82FC-4528-98AE-CEE8214B9C92}"/>
-    <hyperlink ref="I24" r:id="rId22" display="https://kig.pl/wp-content/uploads/2020/07/EN_H2_ENG.pdf" xr:uid="{4AB8A96D-7812-41BE-B837-E2A2D9A34498}"/>
-    <hyperlink ref="I25" r:id="rId23" display="https://www.csis.org/analysis/russias-hydrogen-energy-strategy" xr:uid="{C49418BE-301E-44A4-9387-FB09B9A9BE51}"/>
-    <hyperlink ref="I26" r:id="rId24" display="https://www.csis.org/analysis/saudi-arabias-hydrogen-industrial-strategy" xr:uid="{20A8CE19-B4E4-4F15-8CC9-58F8D122B22E}"/>
-    <hyperlink ref="I27" r:id="rId25" display="https://www.dst.gov.za/images/South_African_Hydrogen_Society_RoadmapV1.pdf" xr:uid="{89E07F63-28E8-4AC5-B933-D07365654E76}"/>
-    <hyperlink ref="I28" r:id="rId26" display="https://energia.gob.es/es-es/Novedades/Documents/hoja_de_ruta_del_hidrogeno.pdf" xr:uid="{8FE55569-3F54-4599-9150-689115558D96}"/>
-    <hyperlink ref="I29" r:id="rId27" display="https://fossilfrittsverige.se/en/start-english/strategies/hydrogen/" xr:uid="{D151024F-F37A-4FA2-A238-4A253B8C9052}"/>
-    <hyperlink ref="I30" r:id="rId28" display="https://www.lexology.com/library/detail.aspx?g=1f5af16e-61e3-4276-8d81-46f6672fe23c" xr:uid="{AC8E2CF7-B73F-4163-9A80-C43D4DB07494}"/>
-    <hyperlink ref="I31" r:id="rId29" display="https://www.oeko.de/fileadmin/oekodoc/GIZ-SPIPA-hydrogen-factsheet-North-African-Countries.pdf" xr:uid="{F4ED3DA7-9A3A-4404-A93F-44D9E15748FA}"/>
-    <hyperlink ref="I32" r:id="rId30" display="not yet" xr:uid="{CE303612-94FD-44C9-A722-07653A46D253}"/>
-    <hyperlink ref="I33" r:id="rId31" display="https://unece.org/sites/default/files/2021-03/Draft Roadmap for production and use of hydrogen in Ukraine_Final .pdf" xr:uid="{4C7D74AC-93FE-4B87-B959-38BCE9FE51DE}"/>
-    <hyperlink ref="I34" r:id="rId32" display="https://www.gub.uy/ministerio-industria-energia-mineria/sites/ministerio-industria-energia-mineria/files/documentos/noticias/Green Hydrogen Roadmap in Uruguay.pdf" xr:uid="{AB940884-964C-4547-B443-EEF954ABDB57}"/>
-    <hyperlink ref="I35" r:id="rId33" display="yes" xr:uid="{68750013-0C74-4946-B9CD-C530418B4198}"/>
-    <hyperlink ref="I36" r:id="rId34" display="https://vietnamnet.vn/en/green-hydrogen-in-the-roadmap-of-energy-transition-in-vietnam-787880.html" xr:uid="{5262637D-2874-41E6-BC6D-5DEB6DB912E2}"/>
+    <hyperlink ref="I25" r:id="rId21" display="https://kig.pl/wp-content/uploads/2020/07/EN_H2_ENG.pdf" xr:uid="{4AB8A96D-7812-41BE-B837-E2A2D9A34498}"/>
+    <hyperlink ref="I26" r:id="rId22" display="https://www.csis.org/analysis/russias-hydrogen-energy-strategy" xr:uid="{C49418BE-301E-44A4-9387-FB09B9A9BE51}"/>
+    <hyperlink ref="I27" r:id="rId23" display="https://www.csis.org/analysis/saudi-arabias-hydrogen-industrial-strategy" xr:uid="{20A8CE19-B4E4-4F15-8CC9-58F8D122B22E}"/>
+    <hyperlink ref="I28" r:id="rId24" display="https://www.dst.gov.za/images/South_African_Hydrogen_Society_RoadmapV1.pdf" xr:uid="{89E07F63-28E8-4AC5-B933-D07365654E76}"/>
+    <hyperlink ref="I29" r:id="rId25" display="https://energia.gob.es/es-es/Novedades/Documents/hoja_de_ruta_del_hidrogeno.pdf" xr:uid="{8FE55569-3F54-4599-9150-689115558D96}"/>
+    <hyperlink ref="I30" r:id="rId26" display="https://fossilfrittsverige.se/en/start-english/strategies/hydrogen/" xr:uid="{D151024F-F37A-4FA2-A238-4A253B8C9052}"/>
+    <hyperlink ref="I31" r:id="rId27" display="https://www.lexology.com/library/detail.aspx?g=1f5af16e-61e3-4276-8d81-46f6672fe23c" xr:uid="{AC8E2CF7-B73F-4163-9A80-C43D4DB07494}"/>
+    <hyperlink ref="I32" r:id="rId28" display="https://www.oeko.de/fileadmin/oekodoc/GIZ-SPIPA-hydrogen-factsheet-North-African-Countries.pdf" xr:uid="{F4ED3DA7-9A3A-4404-A93F-44D9E15748FA}"/>
+    <hyperlink ref="I33" r:id="rId29" display="not yet" xr:uid="{CE303612-94FD-44C9-A722-07653A46D253}"/>
+    <hyperlink ref="I34" r:id="rId30" display="https://unece.org/sites/default/files/2021-03/Draft Roadmap for production and use of hydrogen in Ukraine_Final .pdf" xr:uid="{4C7D74AC-93FE-4B87-B959-38BCE9FE51DE}"/>
+    <hyperlink ref="I35" r:id="rId31" display="https://www.gub.uy/ministerio-industria-energia-mineria/sites/ministerio-industria-energia-mineria/files/documentos/noticias/Green Hydrogen Roadmap in Uruguay.pdf" xr:uid="{AB940884-964C-4547-B443-EEF954ABDB57}"/>
+    <hyperlink ref="I36" r:id="rId32" display="yes" xr:uid="{68750013-0C74-4946-B9CD-C530418B4198}"/>
+    <hyperlink ref="I37" r:id="rId33" display="https://vietnamnet.vn/en/green-hydrogen-in-the-roadmap-of-energy-transition-in-vietnam-787880.html" xr:uid="{5262637D-2874-41E6-BC6D-5DEB6DB912E2}"/>
+    <hyperlink ref="I23" r:id="rId34" display="https://fuelcellsworks.com/news/h2-peru-publishes-its-proposal-for-a-green-hydrogen-roadmap-in-peru/" xr:uid="{93D8A6AB-82FC-4528-98AE-CEE8214B9C92}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId35"/>
@@ -10153,24 +9850,16 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="A54 A28:B31 A3:A4 A7 A5:C6 A49:F49 A26:F26 A52:C52 A33:A49 C28:C49 A8:C27 A50:C50">
-    <cfRule type="expression" dxfId="7" priority="31">
+  <conditionalFormatting sqref="A3:A4 A5:C6 A7 A8:C27 A26:F26 A28:B31 A49:F49 A50:C50 A52:C52 A54">
+    <cfRule type="expression" dxfId="5" priority="31">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
     <cfRule type="expression" priority="32">
       <formula>MOD(COLUMN(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B33:B36">
-    <cfRule type="expression" dxfId="6" priority="29">
-      <formula>MOD(ROW(),2)=0</formula>
-    </cfRule>
-    <cfRule type="expression" priority="30">
-      <formula>MOD(COLUMN(),2)=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="B37:B49">
-    <cfRule type="expression" dxfId="5" priority="27">
+  <conditionalFormatting sqref="A33:B49">
+    <cfRule type="expression" dxfId="4" priority="27">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
     <cfRule type="expression" priority="28">
@@ -10178,23 +9867,23 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6">
-    <cfRule type="expression" dxfId="4" priority="23">
+    <cfRule type="expression" dxfId="3" priority="23">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
     <cfRule type="expression" priority="24">
       <formula>MOD(COLUMN(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C29:C31">
-    <cfRule type="expression" dxfId="3" priority="21">
+  <conditionalFormatting sqref="C11">
+    <cfRule type="expression" dxfId="2" priority="11">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
-    <cfRule type="expression" priority="22">
+    <cfRule type="expression" priority="12">
       <formula>MOD(COLUMN(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C28">
-    <cfRule type="expression" dxfId="2" priority="19">
+  <conditionalFormatting sqref="C28:C49">
+    <cfRule type="expression" dxfId="1" priority="19">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
     <cfRule type="expression" priority="20">
@@ -10202,18 +9891,10 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C53">
-    <cfRule type="expression" dxfId="1" priority="17">
+    <cfRule type="expression" dxfId="0" priority="17">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
     <cfRule type="expression" priority="18">
-      <formula>MOD(COLUMN(),2)=0</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C11">
-    <cfRule type="expression" dxfId="0" priority="11">
-      <formula>MOD(ROW(),2)=0</formula>
-    </cfRule>
-    <cfRule type="expression" priority="12">
       <formula>MOD(COLUMN(),2)=0</formula>
     </cfRule>
   </conditionalFormatting>
@@ -10276,15 +9957,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100E2F0DF90B070FE43BFD707F72A4CD00B" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="8927d14e1bc908eae180c9caa4b5da89">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc94727-11e8-4443-b8f0-9215ff28e4bb" xmlns:ns3="cd34aed5-94da-4c30-bba3-37b78f4daae9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bb67c9392edae2d7a3a1d88d3e91258a" ns2:_="" ns3:_="">
     <xsd:import namespace="1bc94727-11e8-4443-b8f0-9215ff28e4bb"/>
@@ -10521,15 +10193,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22BF5C6F-88A2-47DA-9B5F-9FD29A58E304}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1143ECE1-9C35-446D-8A76-82388033D272}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10546,4 +10219,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22BF5C6F-88A2-47DA-9B5F-9FD29A58E304}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
set "no analysis" for Pakistan RE potential in context data
</commit_message>
<xml_diff>
--- a/data/context_data.xlsx
+++ b/data/context_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j.aschauer\nobackup\ptx-boa\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8B69C056-AA8E-47A1-BE01-EFA89FDB04A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FD4F54-38C1-4BEE-A1FE-A1FC76BD03D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{D16C601B-E1D6-40C0-8CC1-80505BE1FBB6}"/>
   </bookViews>
@@ -7661,10 +7661,10 @@
         <v>654</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>12</v>
+        <v>250</v>
       </c>
       <c r="D23" s="21" t="s">
-        <v>12</v>
+        <v>250</v>
       </c>
       <c r="E23" s="21" t="s">
         <v>12</v>
@@ -8363,8 +8363,8 @@
     <mergeCell ref="C1:D1"/>
     <mergeCell ref="E1:F1"/>
   </mergeCells>
-  <conditionalFormatting sqref="D3:D22 D24:D37">
-    <cfRule type="colorScale" priority="18">
+  <conditionalFormatting sqref="C3:C22 C24:C37">
+    <cfRule type="colorScale" priority="73">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8372,6 +8372,26 @@
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D3:D37">
+    <cfRule type="colorScale" priority="20">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+    <cfRule type="colorScale" priority="23">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E3:E22 E24:E37">
     <cfRule type="colorScale" priority="21">
       <colorScale>
         <cfvo type="min"/>
@@ -8381,8 +8401,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E3:E22 E24:E37">
-    <cfRule type="colorScale" priority="19">
+  <conditionalFormatting sqref="E23">
+    <cfRule type="colorScale" priority="12">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8392,7 +8412,17 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:F22 F24:F37">
-    <cfRule type="colorScale" priority="20">
+    <cfRule type="colorScale" priority="22">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F23">
+    <cfRule type="colorScale" priority="11">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8402,21 +8432,31 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="G3:G37">
-    <cfRule type="cellIs" dxfId="9" priority="12" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="14" operator="equal">
       <formula>"very high"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="8" priority="15" operator="equal">
       <formula>"high"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="16" operator="equal">
       <formula>"medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="17" operator="equal">
       <formula>"low"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="G23">
+    <cfRule type="colorScale" priority="10">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H3:H22 H24:H37">
-    <cfRule type="colorScale" priority="17">
+    <cfRule type="colorScale" priority="19">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -8427,27 +8467,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D23">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E23">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="F23">
+  <conditionalFormatting sqref="H23">
     <cfRule type="colorScale" priority="9">
       <colorScale>
         <cfvo type="min"/>
@@ -8457,7 +8477,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G23">
+  <conditionalFormatting sqref="I23">
     <cfRule type="colorScale" priority="8">
       <colorScale>
         <cfvo type="min"/>
@@ -8467,7 +8487,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H23">
+  <conditionalFormatting sqref="J23">
     <cfRule type="colorScale" priority="7">
       <colorScale>
         <cfvo type="min"/>
@@ -8477,7 +8497,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I23">
+  <conditionalFormatting sqref="K23">
     <cfRule type="colorScale" priority="6">
       <colorScale>
         <cfvo type="min"/>
@@ -8487,7 +8507,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J23">
+  <conditionalFormatting sqref="L23">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -8497,7 +8517,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="K23">
+  <conditionalFormatting sqref="M23">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -8507,7 +8527,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="L23">
+  <conditionalFormatting sqref="N23">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -8517,17 +8537,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="M23">
-    <cfRule type="colorScale" priority="2">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N23">
+  <conditionalFormatting sqref="C23">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -8536,9 +8546,7 @@
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C3:C37">
-    <cfRule type="colorScale" priority="71">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -9957,6 +9965,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100E2F0DF90B070FE43BFD707F72A4CD00B" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="8927d14e1bc908eae180c9caa4b5da89">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc94727-11e8-4443-b8f0-9215ff28e4bb" xmlns:ns3="cd34aed5-94da-4c30-bba3-37b78f4daae9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bb67c9392edae2d7a3a1d88d3e91258a" ns2:_="" ns3:_="">
     <xsd:import namespace="1bc94727-11e8-4443-b8f0-9215ff28e4bb"/>
@@ -10193,16 +10210,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22BF5C6F-88A2-47DA-9B5F-9FD29A58E304}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1143ECE1-9C35-446D-8A76-82388033D272}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10219,12 +10235,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22BF5C6F-88A2-47DA-9B5F-9FD29A58E304}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
add context data for pakistan
</commit_message>
<xml_diff>
--- a/data/context_data.xlsx
+++ b/data/context_data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\j.aschauer\nobackup\ptx-boa\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71FD4F54-38C1-4BEE-A1FE-A1FC76BD03D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8F67714-9270-4795-A07E-047776A9EBBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="2" xr2:uid="{D16C601B-E1D6-40C0-8CC1-80505BE1FBB6}"/>
   </bookViews>
@@ -263,7 +263,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1118" uniqueCount="655">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1114" uniqueCount="656">
   <si>
     <t>topic</t>
   </si>
@@ -2435,6 +2435,9 @@
   </si>
   <si>
     <t>Pakistan</t>
+  </si>
+  <si>
+    <t>not yet [Link](https://www.ppib.gov.pk/news/decarbonization.html)</t>
   </si>
 </sst>
 </file>
@@ -2551,7 +2554,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="48">
+  <cellXfs count="50">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -2694,12 +2697,46 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="1" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Link" xfId="1" builtinId="8"/>
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="34">
+  <dxfs count="38">
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="7" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="9" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <fill>
         <patternFill>
@@ -5829,98 +5866,98 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="J4:J7">
-    <cfRule type="cellIs" dxfId="33" priority="51" operator="equal">
+    <cfRule type="cellIs" dxfId="37" priority="51" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="52" operator="equal">
+    <cfRule type="cellIs" dxfId="36" priority="52" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J11:J15">
-    <cfRule type="cellIs" dxfId="31" priority="5" operator="equal">
+    <cfRule type="cellIs" dxfId="35" priority="5" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="30" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="34" priority="6" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K6:K12">
-    <cfRule type="cellIs" dxfId="29" priority="21" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="21" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="28" priority="22" operator="equal">
+    <cfRule type="cellIs" dxfId="32" priority="22" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K14:K15">
-    <cfRule type="cellIs" dxfId="27" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="31" priority="3" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="26" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="30" priority="4" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L9:L10">
-    <cfRule type="cellIs" dxfId="25" priority="37" operator="equal">
+    <cfRule type="cellIs" dxfId="29" priority="37" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="24" priority="38" operator="equal">
+    <cfRule type="cellIs" dxfId="28" priority="38" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L5:M6">
-    <cfRule type="cellIs" dxfId="23" priority="55" operator="equal">
+    <cfRule type="cellIs" dxfId="27" priority="55" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="22" priority="56" operator="equal">
+    <cfRule type="cellIs" dxfId="26" priority="56" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L12:N12">
-    <cfRule type="cellIs" dxfId="21" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="25" priority="15" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="20" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="24" priority="16" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N6">
-    <cfRule type="cellIs" dxfId="19" priority="53" operator="equal">
+    <cfRule type="cellIs" dxfId="23" priority="53" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="18" priority="54" operator="equal">
+    <cfRule type="cellIs" dxfId="22" priority="54" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O4">
-    <cfRule type="cellIs" dxfId="17" priority="69" operator="equal">
+    <cfRule type="cellIs" dxfId="21" priority="69" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="16" priority="70" operator="equal">
+    <cfRule type="cellIs" dxfId="20" priority="70" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O9">
-    <cfRule type="cellIs" dxfId="15" priority="41" operator="equal">
+    <cfRule type="cellIs" dxfId="19" priority="41" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="14" priority="42" operator="equal">
+    <cfRule type="cellIs" dxfId="18" priority="42" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O11:O12">
-    <cfRule type="cellIs" dxfId="13" priority="13" operator="equal">
+    <cfRule type="cellIs" dxfId="17" priority="13" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="12" priority="14" operator="equal">
+    <cfRule type="cellIs" dxfId="16" priority="14" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="O15">
-    <cfRule type="cellIs" dxfId="11" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="15" priority="1" operator="equal">
       <formula>"no"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="10" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="14" priority="2" operator="equal">
       <formula>"yes"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -7654,46 +7691,46 @@
       </c>
     </row>
     <row r="23" spans="1:14" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A23" s="20" t="s">
+      <c r="A23" s="48" t="s">
         <v>653</v>
       </c>
-      <c r="B23" s="20" t="s">
+      <c r="B23" s="48" t="s">
         <v>654</v>
       </c>
-      <c r="C23" s="21" t="s">
-        <v>250</v>
-      </c>
-      <c r="D23" s="21" t="s">
-        <v>250</v>
-      </c>
-      <c r="E23" s="21" t="s">
+      <c r="C23" s="49">
+        <v>31927</v>
+      </c>
+      <c r="D23" s="49">
+        <v>547</v>
+      </c>
+      <c r="E23" s="49">
+        <v>0</v>
+      </c>
+      <c r="F23" s="49">
+        <v>13</v>
+      </c>
+      <c r="G23" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="F23" s="21" t="s">
+      <c r="H23" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="G23" s="21" t="s">
+      <c r="I23" s="49" t="s">
+        <v>655</v>
+      </c>
+      <c r="J23" s="48" t="s">
+        <v>313</v>
+      </c>
+      <c r="K23" s="48" t="s">
+        <v>318</v>
+      </c>
+      <c r="L23" s="48" t="s">
+        <v>319</v>
+      </c>
+      <c r="M23" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="H23" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="I23" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="J23" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="K23" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="L23" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="M23" s="21" t="s">
-        <v>12</v>
-      </c>
-      <c r="N23" s="21" t="s">
+      <c r="N23" s="49" t="s">
         <v>12</v>
       </c>
     </row>
@@ -8364,7 +8401,7 @@
     <mergeCell ref="E1:F1"/>
   </mergeCells>
   <conditionalFormatting sqref="C3:C22 C24:C37">
-    <cfRule type="colorScale" priority="73">
+    <cfRule type="colorScale" priority="86">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8373,8 +8410,8 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D3:D37">
-    <cfRule type="colorScale" priority="20">
+  <conditionalFormatting sqref="D3:D22 D24:D37">
+    <cfRule type="colorScale" priority="33">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8382,7 +8419,7 @@
         <color rgb="FF63BE7B"/>
       </colorScale>
     </cfRule>
-    <cfRule type="colorScale" priority="23">
+    <cfRule type="colorScale" priority="36">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8392,17 +8429,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="E3:E22 E24:E37">
-    <cfRule type="colorScale" priority="21">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="E23">
-    <cfRule type="colorScale" priority="12">
+    <cfRule type="colorScale" priority="34">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8412,7 +8439,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F3:F22 F24:F37">
-    <cfRule type="colorScale" priority="22">
+    <cfRule type="colorScale" priority="35">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8421,42 +8448,22 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F23">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="G3:G37">
-    <cfRule type="cellIs" dxfId="9" priority="14" operator="equal">
+  <conditionalFormatting sqref="G3:G22 G24:G37">
+    <cfRule type="cellIs" dxfId="13" priority="27" operator="equal">
       <formula>"very high"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="15" operator="equal">
+    <cfRule type="cellIs" dxfId="12" priority="28" operator="equal">
       <formula>"high"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="16" operator="equal">
+    <cfRule type="cellIs" dxfId="11" priority="29" operator="equal">
       <formula>"medium"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="17" operator="equal">
+    <cfRule type="cellIs" dxfId="10" priority="30" operator="equal">
       <formula>"low"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="G23">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <conditionalFormatting sqref="H3:H22 H24:H37">
-    <cfRule type="colorScale" priority="19">
+    <cfRule type="colorScale" priority="32">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="percentile" val="50"/>
@@ -8467,8 +8474,72 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="C23">
+    <cfRule type="colorScale" priority="13">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D23">
+    <cfRule type="colorScale" priority="8">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E23">
+    <cfRule type="colorScale" priority="7">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="F23">
+    <cfRule type="colorScale" priority="6">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G23">
+    <cfRule type="cellIs" dxfId="3" priority="9" operator="equal">
+      <formula>"very high"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="10" operator="equal">
+      <formula>"high"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="11" operator="equal">
+      <formula>"medium"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="12" operator="equal">
+      <formula>"low"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="G23">
+    <cfRule type="colorScale" priority="5">
+      <colorScale>
+        <cfvo type="min"/>
+        <cfvo type="max"/>
+        <color rgb="FFFCFCFF"/>
+        <color rgb="FF63BE7B"/>
+      </colorScale>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="H23">
-    <cfRule type="colorScale" priority="9">
+    <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8478,37 +8549,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="I23">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J23">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K23">
-    <cfRule type="colorScale" priority="6">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L23">
-    <cfRule type="colorScale" priority="5">
+    <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8518,7 +8559,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="M23">
-    <cfRule type="colorScale" priority="4">
+    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8528,25 +8569,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="N23">
-    <cfRule type="colorScale" priority="3">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="C23">
     <cfRule type="colorScale" priority="1">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="max"/>
-        <color rgb="FFFCFCFF"/>
-        <color rgb="FF63BE7B"/>
-      </colorScale>
-    </cfRule>
-    <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
         <cfvo type="max"/>
@@ -8589,7 +8612,7 @@
     <hyperlink ref="I35" r:id="rId31" display="https://www.gub.uy/ministerio-industria-energia-mineria/sites/ministerio-industria-energia-mineria/files/documentos/noticias/Green Hydrogen Roadmap in Uruguay.pdf" xr:uid="{AB940884-964C-4547-B443-EEF954ABDB57}"/>
     <hyperlink ref="I36" r:id="rId32" display="yes" xr:uid="{68750013-0C74-4946-B9CD-C530418B4198}"/>
     <hyperlink ref="I37" r:id="rId33" display="https://vietnamnet.vn/en/green-hydrogen-in-the-roadmap-of-energy-transition-in-vietnam-787880.html" xr:uid="{5262637D-2874-41E6-BC6D-5DEB6DB912E2}"/>
-    <hyperlink ref="I23" r:id="rId34" display="https://fuelcellsworks.com/news/h2-peru-publishes-its-proposal-for-a-green-hydrogen-roadmap-in-peru/" xr:uid="{93D8A6AB-82FC-4528-98AE-CEE8214B9C92}"/>
+    <hyperlink ref="I23" r:id="rId34" display="https://fuelcellsworks.com/news/h2-peru-publishes-its-proposal-for-a-green-hydrogen-roadmap-in-peru/" xr:uid="{4E0DB980-714D-493C-9BDC-37103EA3004E}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId35"/>
@@ -9859,7 +9882,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="A3:A4 A5:C6 A7 A8:C27 A26:F26 A28:B31 A49:F49 A50:C50 A52:C52 A54">
-    <cfRule type="expression" dxfId="5" priority="31">
+    <cfRule type="expression" dxfId="9" priority="31">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
     <cfRule type="expression" priority="32">
@@ -9867,7 +9890,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="A33:B49">
-    <cfRule type="expression" dxfId="4" priority="27">
+    <cfRule type="expression" dxfId="8" priority="27">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
     <cfRule type="expression" priority="28">
@@ -9875,7 +9898,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C6">
-    <cfRule type="expression" dxfId="3" priority="23">
+    <cfRule type="expression" dxfId="7" priority="23">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
     <cfRule type="expression" priority="24">
@@ -9883,7 +9906,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C11">
-    <cfRule type="expression" dxfId="2" priority="11">
+    <cfRule type="expression" dxfId="6" priority="11">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
     <cfRule type="expression" priority="12">
@@ -9891,7 +9914,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C28:C49">
-    <cfRule type="expression" dxfId="1" priority="19">
+    <cfRule type="expression" dxfId="5" priority="19">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
     <cfRule type="expression" priority="20">
@@ -9899,7 +9922,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C53">
-    <cfRule type="expression" dxfId="0" priority="17">
+    <cfRule type="expression" dxfId="4" priority="17">
       <formula>MOD(ROW(),2)=0</formula>
     </cfRule>
     <cfRule type="expression" priority="18">
@@ -9965,15 +9988,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Dokument" ma:contentTypeID="0x010100E2F0DF90B070FE43BFD707F72A4CD00B" ma:contentTypeVersion="15" ma:contentTypeDescription="Ein neues Dokument erstellen." ma:contentTypeScope="" ma:versionID="8927d14e1bc908eae180c9caa4b5da89">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="1bc94727-11e8-4443-b8f0-9215ff28e4bb" xmlns:ns3="cd34aed5-94da-4c30-bba3-37b78f4daae9" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="bb67c9392edae2d7a3a1d88d3e91258a" ns2:_="" ns3:_="">
     <xsd:import namespace="1bc94727-11e8-4443-b8f0-9215ff28e4bb"/>
@@ -10210,15 +10224,16 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22BF5C6F-88A2-47DA-9B5F-9FD29A58E304}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1143ECE1-9C35-446D-8A76-82388033D272}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10235,4 +10250,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{22BF5C6F-88A2-47DA-9B5F-9FD29A58E304}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>